<commit_message>
bulkImport: slim templates to match existing admin forms
Drops vestigial columns the existing UI never sets:
- components: removed value (no input in admin form), min_stock_level,
  reorder_point, warehouse_location, vendor_id, image_2..5, video_url
- products: removed vendor_id, image_2..5, video_url
- Both now have one image_url column instead of 5 + a video column

Templates now mirror the actual admin form fields 1:1. Components are
9 columns, products are 8 columns.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/components-import-template.xlsx
+++ b/public/templates/components-import-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -411,52 +411,22 @@
         <v>type</v>
       </c>
       <c r="D1" t="str">
-        <v>value</v>
+        <v>description</v>
       </c>
       <c r="E1" t="str">
-        <v>description</v>
+        <v>normal_price</v>
       </c>
       <c r="F1" t="str">
-        <v>normal_price</v>
+        <v>merchant_price</v>
       </c>
       <c r="G1" t="str">
-        <v>merchant_price</v>
+        <v>stock_level</v>
       </c>
       <c r="H1" t="str">
-        <v>stock_level</v>
+        <v>is_active</v>
       </c>
       <c r="I1" t="str">
-        <v>min_stock_level</v>
-      </c>
-      <c r="J1" t="str">
-        <v>reorder_point</v>
-      </c>
-      <c r="K1" t="str">
-        <v>warehouse_location</v>
-      </c>
-      <c r="L1" t="str">
-        <v>is_active</v>
-      </c>
-      <c r="M1" t="str">
-        <v>vendor_id</v>
-      </c>
-      <c r="N1" t="str">
-        <v>image_1</v>
-      </c>
-      <c r="O1" t="str">
-        <v>image_2</v>
-      </c>
-      <c r="P1" t="str">
-        <v>image_3</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>image_4</v>
-      </c>
-      <c r="R1" t="str">
-        <v>image_5</v>
-      </c>
-      <c r="S1" t="str">
-        <v>video_url</v>
+        <v>image_url</v>
       </c>
     </row>
     <row r="2">
@@ -470,64 +440,34 @@
         <v>body</v>
       </c>
       <c r="D2" t="str">
-        <v>M8</v>
-      </c>
-      <c r="E2" t="str">
         <v>Heavy-duty stainless steel bracket</v>
       </c>
+      <c r="E2">
+        <v>12.5</v>
+      </c>
       <c r="F2">
-        <v>12.5</v>
+        <v>9.8</v>
       </c>
       <c r="G2">
-        <v>9.8</v>
-      </c>
-      <c r="H2">
         <v>25</v>
       </c>
-      <c r="I2">
-        <v>10</v>
-      </c>
-      <c r="J2">
-        <v>15</v>
-      </c>
-      <c r="K2" t="str">
-        <v>A1-03</v>
-      </c>
-      <c r="L2" t="str">
+      <c r="H2" t="str">
         <v>TRUE</v>
       </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
+      <c r="I2" t="str">
         <v>https://drive.google.com/file/d/EXAMPLE_FILE_ID/view</v>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-      <c r="S2" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -587,7 +527,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>value</v>
+        <v>description</v>
       </c>
       <c r="B5" t="str">
         <v>no</v>
@@ -601,21 +541,21 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>description</v>
+        <v>normal_price</v>
       </c>
       <c r="B6" t="str">
-        <v>no</v>
+        <v>YES</v>
       </c>
       <c r="C6" t="str">
-        <v>text</v>
+        <v>number</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>min: 0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>normal_price</v>
+        <v>merchant_price</v>
       </c>
       <c r="B7" t="str">
         <v>YES</v>
@@ -629,13 +569,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>merchant_price</v>
+        <v>stock_level</v>
       </c>
       <c r="B8" t="str">
-        <v>YES</v>
+        <v>no</v>
       </c>
       <c r="C8" t="str">
-        <v>number</v>
+        <v>integer</v>
       </c>
       <c r="D8" t="str">
         <v>min: 0</v>
@@ -643,217 +583,77 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>stock_level</v>
+        <v>is_active</v>
       </c>
       <c r="B9" t="str">
         <v>no</v>
       </c>
       <c r="C9" t="str">
-        <v>integer</v>
+        <v>boolean</v>
       </c>
       <c r="D9" t="str">
-        <v>min: 0</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>min_stock_level</v>
+        <v>image_url</v>
       </c>
       <c r="B10" t="str">
         <v>no</v>
       </c>
       <c r="C10" t="str">
-        <v>integer</v>
+        <v>url</v>
       </c>
       <c r="D10" t="str">
-        <v>min: 0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>reorder_point</v>
-      </c>
-      <c r="B11" t="str">
-        <v>no</v>
-      </c>
-      <c r="C11" t="str">
-        <v>integer</v>
-      </c>
-      <c r="D11" t="str">
-        <v>min: 0</v>
+        <v>Drive share URL or any https URL — re-hosted on import</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>warehouse_location</v>
+        <v>Drive sharing required</v>
       </c>
       <c r="B12" t="str">
-        <v>no</v>
+        <v/>
       </c>
       <c r="C12" t="str">
-        <v>text</v>
+        <v/>
       </c>
       <c r="D12" t="str">
-        <v/>
+        <v>Right-click folder → Share → "Anyone with the link"</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>is_active</v>
+        <v>Image size cap</v>
       </c>
       <c r="B13" t="str">
-        <v>no</v>
+        <v/>
       </c>
       <c r="C13" t="str">
-        <v>boolean</v>
+        <v/>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>Keep files under 25 MB to avoid Drive virus-scan interstitial</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>vendor_id</v>
+        <v>Boolean values</v>
       </c>
       <c r="B14" t="str">
-        <v>no</v>
+        <v/>
       </c>
       <c r="C14" t="str">
-        <v>uuid</v>
+        <v/>
       </c>
       <c r="D14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>image_1</v>
-      </c>
-      <c r="B15" t="str">
-        <v>no</v>
-      </c>
-      <c r="C15" t="str">
-        <v>url</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Drive share URL or any https URL — re-hosted on import</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>image_2</v>
-      </c>
-      <c r="B16" t="str">
-        <v>no</v>
-      </c>
-      <c r="C16" t="str">
-        <v>url</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Drive share URL or any https URL — re-hosted on import</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>image_3</v>
-      </c>
-      <c r="B17" t="str">
-        <v>no</v>
-      </c>
-      <c r="C17" t="str">
-        <v>url</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Drive share URL or any https URL — re-hosted on import</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>image_4</v>
-      </c>
-      <c r="B18" t="str">
-        <v>no</v>
-      </c>
-      <c r="C18" t="str">
-        <v>url</v>
-      </c>
-      <c r="D18" t="str">
-        <v>Drive share URL or any https URL — re-hosted on import</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>image_5</v>
-      </c>
-      <c r="B19" t="str">
-        <v>no</v>
-      </c>
-      <c r="C19" t="str">
-        <v>url</v>
-      </c>
-      <c r="D19" t="str">
-        <v>Drive share URL or any https URL — re-hosted on import</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>video_url</v>
-      </c>
-      <c r="B20" t="str">
-        <v>no</v>
-      </c>
-      <c r="C20" t="str">
-        <v>url</v>
-      </c>
-      <c r="D20" t="str">
-        <v>YouTube/Vimeo/Drive — stored as-is</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Drive sharing required</v>
-      </c>
-      <c r="B22" t="str">
-        <v/>
-      </c>
-      <c r="C22" t="str">
-        <v/>
-      </c>
-      <c r="D22" t="str">
-        <v>Right-click folder → Share → "Anyone with the link"</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Image size cap</v>
-      </c>
-      <c r="B23" t="str">
-        <v/>
-      </c>
-      <c r="C23" t="str">
-        <v/>
-      </c>
-      <c r="D23" t="str">
-        <v>Keep files under 25 MB to avoid Drive virus-scan interstitial</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Boolean values</v>
-      </c>
-      <c r="B24" t="str">
-        <v/>
-      </c>
-      <c r="C24" t="str">
-        <v/>
-      </c>
-      <c r="D24" t="str">
         <v>TRUE / FALSE / yes / no / 1 / 0 all accepted</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>